<commit_message>
docs: update documentation and time table
</commit_message>
<xml_diff>
--- a/docs/JIPA_Nikola_Zeitplan.xlsx
+++ b/docs/JIPA_Nikola_Zeitplan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NikolaManojlovic\Desktop\JIPA Vorbereitung\JIPA Nikola\Code\jipa-pflanzen-app\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aspergerinf-my.sharepoint.com/personal/nikola_manojlovic_twofold_swiss/Documents/JIPA Vorbereitung/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{587A545B-0971-4973-AAA7-E747BA1DE290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB225FD7-DFDE-4183-9B20-29F2B23DB61B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30612" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,13 +41,82 @@
     <t>Aufgabe</t>
   </si>
   <si>
-    <t>Informieren</t>
+    <t>Zeitaufwand (h)</t>
+  </si>
+  <si>
+    <t>Soll</t>
+  </si>
+  <si>
+    <t>Ist</t>
+  </si>
+  <si>
+    <t>Allgemeines</t>
+  </si>
+  <si>
+    <t>Legende</t>
+  </si>
+  <si>
+    <t>Versionierung aufsetzen</t>
+  </si>
+  <si>
+    <t>1. Meilenstein (IPE-Abschluss)</t>
+  </si>
+  <si>
+    <t>2. Meilenstein (R-Abschluss)</t>
+  </si>
+  <si>
+    <t>Projektgrundlagen einrichten</t>
+  </si>
+  <si>
+    <t>3. Meilenstein (K-Abschluss)</t>
+  </si>
+  <si>
+    <t>4. Meilenstein (A-Abschluss)</t>
   </si>
   <si>
     <t>Zeitplan erstellen</t>
   </si>
   <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Dokumentation</t>
+  </si>
+  <si>
+    <t>Arbeitsjournal führen</t>
+  </si>
+  <si>
+    <t>Expertenbesuch</t>
+  </si>
+  <si>
+    <t>Puffer</t>
+  </si>
+  <si>
+    <t>Informieren</t>
+  </si>
+  <si>
+    <t>Dokumentation Teil 1</t>
+  </si>
+  <si>
+    <t>Kurzfassung &amp; Informieren</t>
+  </si>
+  <si>
+    <t>Anforderungsanalyse</t>
+  </si>
+  <si>
     <t>Planen</t>
+  </si>
+  <si>
+    <t>Kernfeatures Planen</t>
+  </si>
+  <si>
+    <t>Testkonzept erstellen</t>
+  </si>
+  <si>
+    <t>Diagramme</t>
+  </si>
+  <si>
+    <t>Datenbank</t>
   </si>
   <si>
     <t>Entscheiden</t>
@@ -57,6 +126,24 @@
   </si>
   <si>
     <t>Realisieren</t>
+  </si>
+  <si>
+    <t>Projekt &amp; Datenbankerstellung</t>
+  </si>
+  <si>
+    <t>Pflanzen Endpunkte</t>
+  </si>
+  <si>
+    <t>Giessen Endpunkte</t>
+  </si>
+  <si>
+    <t>Kategorie Endpunkte</t>
+  </si>
+  <si>
+    <t>Validierung &amp; Fehlerbehandlung</t>
+  </si>
+  <si>
+    <t>Swagger Dokumentation</t>
   </si>
   <si>
     <t>Kontrollieren</t>
@@ -74,101 +161,14 @@
     <t>Gesamtprojektauswertung</t>
   </si>
   <si>
-    <t>Legende</t>
-  </si>
-  <si>
-    <t>1. Meilenstein (IPE-Abschluss)</t>
-  </si>
-  <si>
-    <t>2. Meilenstein (R-Abschluss)</t>
-  </si>
-  <si>
-    <t>3. Meilenstein (K-Abschluss)</t>
-  </si>
-  <si>
-    <t>4. Meilenstein (A-Abschluss)</t>
-  </si>
-  <si>
-    <t>Soll</t>
-  </si>
-  <si>
-    <t>Ist</t>
-  </si>
-  <si>
-    <t>Zeitaufwand (h)</t>
-  </si>
-  <si>
-    <t>Puffer</t>
-  </si>
-  <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>Arbeitsjournal führen</t>
-  </si>
-  <si>
-    <t>Dokumentation</t>
-  </si>
-  <si>
-    <t>Versionierung aufsetzen</t>
-  </si>
-  <si>
-    <t>Anforderungsanalyse</t>
-  </si>
-  <si>
-    <t>Expertenbesuch</t>
-  </si>
-  <si>
-    <t>Testkonzept erstellen</t>
-  </si>
-  <si>
-    <t>Kernfeatures Planen</t>
-  </si>
-  <si>
-    <t>Dokumentation Teil 1</t>
-  </si>
-  <si>
-    <t>Kurzfassung &amp; Informieren</t>
-  </si>
-  <si>
-    <t>Diagramme</t>
-  </si>
-  <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t>Datenbank</t>
-  </si>
-  <si>
-    <t>Allgemeines</t>
-  </si>
-  <si>
-    <t>Projekt &amp; Datenbankerstellung</t>
-  </si>
-  <si>
-    <t>Pflanzen Endpunkte</t>
-  </si>
-  <si>
-    <t>Giessen Endpunkte</t>
-  </si>
-  <si>
-    <t>Kategorie Endpunkte</t>
-  </si>
-  <si>
-    <t>Swagger Dokumentation</t>
-  </si>
-  <si>
-    <t>Validierung &amp; Fehlerbehandlung</t>
-  </si>
-  <si>
-    <t>Projektgrundlagen einrichten</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1171,14 +1171,82 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1186,12 +1254,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1211,75 +1273,13 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1304,14 +1304,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1349,7 +1345,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1455,7 +1451,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1597,7 +1593,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1606,7 +1602,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:OT128"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="24.95" customHeight="1" thickTop="1" thickBottom="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="24.95" customHeight="1" thickTop="1" thickBottom="1"/>
   <cols>
     <col min="1" max="1" width="6.85546875" style="82" customWidth="1"/>
     <col min="2" max="2" width="28.7109375" style="20" customWidth="1"/>
@@ -1626,7 +1622,7 @@
     <col min="538" max="538" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:410" s="10" customFormat="1" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:410" s="10" customFormat="1" ht="37.5" customHeight="1" thickBot="1">
       <c r="A1" s="13"/>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -1672,75 +1668,75 @@
       <c r="AQ1" s="13"/>
       <c r="AR1" s="13"/>
     </row>
-    <row r="2" spans="1:410" s="7" customFormat="1" ht="29.45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:410" s="7" customFormat="1" ht="29.45" customHeight="1" thickTop="1" thickBot="1">
       <c r="A2" s="10"/>
       <c r="B2" s="83" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="129" t="s">
-        <v>19</v>
+      <c r="C2" s="125" t="s">
+        <v>1</v>
       </c>
-      <c r="D2" s="130"/>
-      <c r="E2" s="124">
+      <c r="D2" s="126"/>
+      <c r="E2" s="118">
         <v>46300</v>
       </c>
-      <c r="F2" s="125"/>
-      <c r="G2" s="125"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="124">
+      <c r="F2" s="119"/>
+      <c r="G2" s="119"/>
+      <c r="H2" s="120"/>
+      <c r="I2" s="118">
         <v>46301</v>
       </c>
-      <c r="J2" s="125"/>
-      <c r="K2" s="125"/>
-      <c r="L2" s="127"/>
-      <c r="M2" s="124">
+      <c r="J2" s="119"/>
+      <c r="K2" s="119"/>
+      <c r="L2" s="120"/>
+      <c r="M2" s="118">
         <v>46302</v>
       </c>
-      <c r="N2" s="125"/>
-      <c r="O2" s="125"/>
-      <c r="P2" s="127"/>
-      <c r="Q2" s="124">
+      <c r="N2" s="119"/>
+      <c r="O2" s="119"/>
+      <c r="P2" s="120"/>
+      <c r="Q2" s="118">
         <v>46303</v>
       </c>
-      <c r="R2" s="125"/>
-      <c r="S2" s="125"/>
-      <c r="T2" s="127"/>
-      <c r="U2" s="124">
+      <c r="R2" s="119"/>
+      <c r="S2" s="119"/>
+      <c r="T2" s="120"/>
+      <c r="U2" s="118">
         <v>46304</v>
       </c>
-      <c r="V2" s="125"/>
-      <c r="W2" s="125"/>
-      <c r="X2" s="127"/>
-      <c r="Y2" s="124">
+      <c r="V2" s="119"/>
+      <c r="W2" s="119"/>
+      <c r="X2" s="120"/>
+      <c r="Y2" s="118">
         <v>46307</v>
       </c>
-      <c r="Z2" s="125"/>
-      <c r="AA2" s="125"/>
-      <c r="AB2" s="127"/>
-      <c r="AC2" s="124">
+      <c r="Z2" s="119"/>
+      <c r="AA2" s="119"/>
+      <c r="AB2" s="120"/>
+      <c r="AC2" s="118">
         <v>46308</v>
       </c>
-      <c r="AD2" s="125"/>
-      <c r="AE2" s="125"/>
-      <c r="AF2" s="127"/>
-      <c r="AG2" s="124">
+      <c r="AD2" s="119"/>
+      <c r="AE2" s="119"/>
+      <c r="AF2" s="120"/>
+      <c r="AG2" s="118">
         <v>46309</v>
       </c>
-      <c r="AH2" s="125"/>
-      <c r="AI2" s="125"/>
-      <c r="AJ2" s="127"/>
-      <c r="AK2" s="124">
+      <c r="AH2" s="119"/>
+      <c r="AI2" s="119"/>
+      <c r="AJ2" s="120"/>
+      <c r="AK2" s="118">
         <v>46310</v>
       </c>
-      <c r="AL2" s="125"/>
-      <c r="AM2" s="125"/>
-      <c r="AN2" s="125"/>
-      <c r="AO2" s="124">
+      <c r="AL2" s="119"/>
+      <c r="AM2" s="119"/>
+      <c r="AN2" s="119"/>
+      <c r="AO2" s="118">
         <v>46311</v>
       </c>
-      <c r="AP2" s="125"/>
-      <c r="AQ2" s="125"/>
-      <c r="AR2" s="126"/>
+      <c r="AP2" s="119"/>
+      <c r="AQ2" s="119"/>
+      <c r="AR2" s="123"/>
       <c r="AS2" s="14"/>
       <c r="AT2" s="14"/>
       <c r="AU2" s="14"/>
@@ -2108,14 +2104,14 @@
       <c r="OS2" s="80"/>
       <c r="OT2" s="81"/>
     </row>
-    <row r="3" spans="1:410" s="7" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:410" s="7" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A3" s="10"/>
       <c r="B3" s="59"/>
       <c r="C3" s="42" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E3" s="85">
         <v>2</v>
@@ -2238,8 +2234,8 @@
         <v>8</v>
       </c>
       <c r="AS3" s="14"/>
-      <c r="AT3" s="135"/>
-      <c r="AU3" s="135"/>
+      <c r="AT3" s="109"/>
+      <c r="AU3" s="109"/>
       <c r="AV3" s="14"/>
       <c r="AW3" s="14"/>
       <c r="AX3" s="14"/>
@@ -2604,10 +2600,10 @@
       <c r="OS3" s="6"/>
       <c r="OT3" s="6"/>
     </row>
-    <row r="4" spans="1:410" s="7" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:410" s="7" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A4" s="10"/>
       <c r="B4" s="84" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="E4" s="70"/>
       <c r="F4" s="70"/>
@@ -2650,10 +2646,10 @@
       <c r="AQ4" s="70"/>
       <c r="AR4" s="72"/>
       <c r="AS4" s="14"/>
-      <c r="AT4" s="133" t="s">
-        <v>12</v>
+      <c r="AT4" s="107" t="s">
+        <v>5</v>
       </c>
-      <c r="AU4" s="134"/>
+      <c r="AU4" s="108"/>
       <c r="AV4" s="14"/>
       <c r="AW4" s="14"/>
       <c r="AX4" s="14"/>
@@ -3018,15 +3014,15 @@
       <c r="OS4" s="6"/>
       <c r="OT4" s="6"/>
     </row>
-    <row r="5" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="105"/>
-      <c r="B5" s="121" t="s">
-        <v>24</v>
+    <row r="5" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A5" s="141"/>
+      <c r="B5" s="114" t="s">
+        <v>6</v>
       </c>
-      <c r="C5" s="139">
+      <c r="C5" s="116">
         <v>2</v>
       </c>
-      <c r="D5" s="121">
+      <c r="D5" s="114">
         <v>0</v>
       </c>
       <c r="E5" s="90">
@@ -3076,7 +3072,7 @@
         <v>1</v>
       </c>
       <c r="AU5" s="38" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="AV5" s="13"/>
       <c r="AW5" s="13"/>
@@ -3436,11 +3432,11 @@
       <c r="OM5" s="4"/>
       <c r="ON5" s="4"/>
     </row>
-    <row r="6" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="105"/>
-      <c r="B6" s="122"/>
-      <c r="C6" s="139"/>
-      <c r="D6" s="128"/>
+    <row r="6" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A6" s="141"/>
+      <c r="B6" s="115"/>
+      <c r="C6" s="116"/>
+      <c r="D6" s="117"/>
       <c r="E6" s="102">
         <v>2</v>
       </c>
@@ -3488,7 +3484,7 @@
         <v>2</v>
       </c>
       <c r="AU6" s="38" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="AV6" s="13"/>
       <c r="AW6" s="13"/>
@@ -3848,15 +3844,15 @@
       <c r="OM6" s="4"/>
       <c r="ON6" s="4"/>
     </row>
-    <row r="7" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="105"/>
-      <c r="B7" s="121" t="s">
-        <v>41</v>
+    <row r="7" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A7" s="141"/>
+      <c r="B7" s="114" t="s">
+        <v>9</v>
       </c>
-      <c r="C7" s="131">
+      <c r="C7" s="121">
         <v>2</v>
       </c>
-      <c r="D7" s="121"/>
+      <c r="D7" s="114"/>
       <c r="E7" s="101">
         <v>2</v>
       </c>
@@ -3904,7 +3900,7 @@
         <v>3</v>
       </c>
       <c r="AU7" s="38" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AV7" s="13"/>
       <c r="AW7" s="13"/>
@@ -4264,11 +4260,11 @@
       <c r="OM7" s="4"/>
       <c r="ON7" s="4"/>
     </row>
-    <row r="8" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="105"/>
-      <c r="B8" s="122"/>
-      <c r="C8" s="132"/>
-      <c r="D8" s="122"/>
+    <row r="8" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A8" s="141"/>
+      <c r="B8" s="115"/>
+      <c r="C8" s="122"/>
+      <c r="D8" s="115"/>
       <c r="E8" s="102">
         <v>2.5</v>
       </c>
@@ -4316,7 +4312,7 @@
         <v>4</v>
       </c>
       <c r="AU8" s="38" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="AV8" s="13"/>
       <c r="AW8" s="13"/>
@@ -4676,15 +4672,15 @@
       <c r="OM8" s="4"/>
       <c r="ON8" s="4"/>
     </row>
-    <row r="9" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="105"/>
-      <c r="B9" s="121" t="s">
-        <v>2</v>
+    <row r="9" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A9" s="141"/>
+      <c r="B9" s="114" t="s">
+        <v>12</v>
       </c>
-      <c r="C9" s="121">
+      <c r="C9" s="114">
         <v>1</v>
       </c>
-      <c r="D9" s="128">
+      <c r="D9" s="117">
         <v>0</v>
       </c>
       <c r="E9" s="51"/>
@@ -4731,10 +4727,10 @@
       <c r="AR9" s="58"/>
       <c r="AS9" s="13"/>
       <c r="AT9" s="39" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="AU9" s="38" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="AV9" s="13"/>
       <c r="AW9" s="13"/>
@@ -5094,11 +5090,11 @@
       <c r="OM9" s="4"/>
       <c r="ON9" s="4"/>
     </row>
-    <row r="10" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="105"/>
-      <c r="B10" s="122"/>
-      <c r="C10" s="122"/>
-      <c r="D10" s="122"/>
+    <row r="10" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A10" s="141"/>
+      <c r="B10" s="115"/>
+      <c r="C10" s="115"/>
+      <c r="D10" s="115"/>
       <c r="E10" s="51"/>
       <c r="F10" s="102">
         <v>0.5</v>
@@ -5143,10 +5139,10 @@
       <c r="AR10" s="58"/>
       <c r="AS10" s="13"/>
       <c r="AT10" s="62" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="AU10" s="38" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="AV10" s="13"/>
       <c r="AW10" s="13"/>
@@ -5506,15 +5502,15 @@
       <c r="OM10" s="4"/>
       <c r="ON10" s="4"/>
     </row>
-    <row r="11" spans="1:410" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="105"/>
-      <c r="B11" s="121" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="121">
+    <row r="11" spans="1:410" ht="12.95" customHeight="1" thickTop="1">
+      <c r="A11" s="141"/>
+      <c r="B11" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="121">
+      <c r="C11" s="114">
+        <v>14</v>
+      </c>
+      <c r="D11" s="114">
         <v>0</v>
       </c>
       <c r="E11" s="51"/>
@@ -5938,11 +5934,11 @@
       <c r="OM11" s="4"/>
       <c r="ON11" s="4"/>
     </row>
-    <row r="12" spans="1:410" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="105"/>
-      <c r="B12" s="122"/>
-      <c r="C12" s="122"/>
-      <c r="D12" s="122"/>
+    <row r="12" spans="1:410" ht="12.95" customHeight="1" thickBot="1">
+      <c r="A12" s="141"/>
+      <c r="B12" s="115"/>
+      <c r="C12" s="115"/>
+      <c r="D12" s="115"/>
       <c r="E12" s="51"/>
       <c r="F12" s="102">
         <v>1</v>
@@ -6346,15 +6342,15 @@
       <c r="OM12" s="4"/>
       <c r="ON12" s="4"/>
     </row>
-    <row r="13" spans="1:410" s="1" customFormat="1" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:410" s="1" customFormat="1" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A13" s="10"/>
-      <c r="B13" s="138" t="s">
-        <v>22</v>
+      <c r="B13" s="113" t="s">
+        <v>15</v>
       </c>
-      <c r="C13" s="121">
+      <c r="C13" s="114">
         <v>4</v>
       </c>
-      <c r="D13" s="121">
+      <c r="D13" s="114">
         <v>0</v>
       </c>
       <c r="E13" s="51"/>
@@ -6784,11 +6780,11 @@
       <c r="OS13" s="2"/>
       <c r="OT13" s="2"/>
     </row>
-    <row r="14" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="105"/>
-      <c r="B14" s="138"/>
-      <c r="C14" s="122"/>
-      <c r="D14" s="122"/>
+    <row r="14" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A14" s="141"/>
+      <c r="B14" s="113"/>
+      <c r="C14" s="115"/>
+      <c r="D14" s="115"/>
       <c r="E14" s="51"/>
       <c r="F14" s="51"/>
       <c r="G14" s="51"/>
@@ -7192,15 +7188,15 @@
       <c r="OM14" s="4"/>
       <c r="ON14" s="4"/>
     </row>
-    <row r="15" spans="1:410" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="105"/>
-      <c r="B15" s="121" t="s">
-        <v>26</v>
+    <row r="15" spans="1:410" ht="12.95" customHeight="1" thickTop="1">
+      <c r="A15" s="141"/>
+      <c r="B15" s="114" t="s">
+        <v>16</v>
       </c>
-      <c r="C15" s="121">
+      <c r="C15" s="114">
         <v>0</v>
       </c>
-      <c r="D15" s="121">
+      <c r="D15" s="114">
         <v>0</v>
       </c>
       <c r="E15" s="51"/>
@@ -7604,11 +7600,11 @@
       <c r="OM15" s="4"/>
       <c r="ON15" s="4"/>
     </row>
-    <row r="16" spans="1:410" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="105"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
+    <row r="16" spans="1:410" ht="12.95" customHeight="1" thickBot="1">
+      <c r="A16" s="141"/>
+      <c r="B16" s="115"/>
+      <c r="C16" s="115"/>
+      <c r="D16" s="115"/>
       <c r="E16" s="51"/>
       <c r="F16" s="51"/>
       <c r="G16" s="51"/>
@@ -8010,15 +8006,15 @@
       <c r="OM16" s="4"/>
       <c r="ON16" s="4"/>
     </row>
-    <row r="17" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="105"/>
-      <c r="B17" s="121" t="s">
-        <v>20</v>
+    <row r="17" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A17" s="141"/>
+      <c r="B17" s="114" t="s">
+        <v>17</v>
       </c>
-      <c r="C17" s="139">
+      <c r="C17" s="116">
         <v>0</v>
       </c>
-      <c r="D17" s="139">
+      <c r="D17" s="116">
         <v>0</v>
       </c>
       <c r="E17" s="51"/>
@@ -8422,11 +8418,11 @@
       <c r="OM17" s="4"/>
       <c r="ON17" s="4"/>
     </row>
-    <row r="18" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="105"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="139"/>
-      <c r="D18" s="139"/>
+    <row r="18" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A18" s="141"/>
+      <c r="B18" s="115"/>
+      <c r="C18" s="116"/>
+      <c r="D18" s="116"/>
       <c r="E18" s="51"/>
       <c r="F18" s="51"/>
       <c r="G18" s="51"/>
@@ -8828,10 +8824,10 @@
       <c r="OM18" s="4"/>
       <c r="ON18" s="4"/>
     </row>
-    <row r="19" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="105"/>
+    <row r="19" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A19" s="141"/>
       <c r="B19" s="61" t="s">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C19" s="32"/>
       <c r="D19" s="33"/>
@@ -9236,15 +9232,15 @@
       <c r="OM19" s="4"/>
       <c r="ON19" s="4"/>
     </row>
-    <row r="20" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="105"/>
-      <c r="B20" s="123" t="s">
-        <v>29</v>
+    <row r="20" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A20" s="141"/>
+      <c r="B20" s="124" t="s">
+        <v>19</v>
       </c>
-      <c r="C20" s="123">
+      <c r="C20" s="124">
         <v>3</v>
       </c>
-      <c r="D20" s="123">
+      <c r="D20" s="124">
         <v>0</v>
       </c>
       <c r="E20" s="67"/>
@@ -9652,11 +9648,11 @@
       <c r="OM20" s="4"/>
       <c r="ON20" s="4"/>
     </row>
-    <row r="21" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="105"/>
-      <c r="B21" s="123"/>
-      <c r="C21" s="123"/>
-      <c r="D21" s="123"/>
+    <row r="21" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A21" s="141"/>
+      <c r="B21" s="124"/>
+      <c r="C21" s="124"/>
+      <c r="D21" s="124"/>
       <c r="E21" s="67"/>
       <c r="F21" s="67"/>
       <c r="G21" s="103">
@@ -9665,9 +9661,9 @@
       <c r="H21" s="104"/>
       <c r="I21" s="103"/>
       <c r="J21" s="103"/>
-      <c r="K21" s="140"/>
-      <c r="L21" s="140"/>
-      <c r="M21" s="140">
+      <c r="K21" s="105"/>
+      <c r="L21" s="105"/>
+      <c r="M21" s="105">
         <v>1.5</v>
       </c>
       <c r="N21" s="50"/>
@@ -10062,15 +10058,15 @@
       <c r="OM21" s="4"/>
       <c r="ON21" s="4"/>
     </row>
-    <row r="22" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="105"/>
-      <c r="B22" s="123" t="s">
-        <v>30</v>
+    <row r="22" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A22" s="141"/>
+      <c r="B22" s="124" t="s">
+        <v>20</v>
       </c>
-      <c r="C22" s="123">
+      <c r="C22" s="124">
         <v>2</v>
       </c>
-      <c r="D22" s="123">
+      <c r="D22" s="124">
         <v>0</v>
       </c>
       <c r="E22" s="67"/>
@@ -10478,11 +10474,11 @@
       <c r="OM22" s="4"/>
       <c r="ON22" s="4"/>
     </row>
-    <row r="23" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="105"/>
-      <c r="B23" s="123"/>
-      <c r="C23" s="123"/>
-      <c r="D23" s="123"/>
+    <row r="23" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A23" s="141"/>
+      <c r="B23" s="124"/>
+      <c r="C23" s="124"/>
+      <c r="D23" s="124"/>
       <c r="E23" s="47"/>
       <c r="F23" s="47"/>
       <c r="G23" s="47"/>
@@ -10491,21 +10487,27 @@
       <c r="J23" s="52"/>
       <c r="K23" s="53"/>
       <c r="L23" s="53"/>
-      <c r="M23" s="141">
+      <c r="M23" s="106">
         <v>0.5</v>
       </c>
-      <c r="N23" s="141">
+      <c r="N23" s="106">
         <v>2</v>
       </c>
-      <c r="O23" s="141">
+      <c r="O23" s="106">
         <v>2</v>
       </c>
-      <c r="P23" s="141">
+      <c r="P23" s="106">
         <v>2</v>
       </c>
-      <c r="Q23" s="53"/>
-      <c r="R23" s="53"/>
-      <c r="S23" s="53"/>
+      <c r="Q23" s="106">
+        <v>2</v>
+      </c>
+      <c r="R23" s="106">
+        <v>2</v>
+      </c>
+      <c r="S23" s="106">
+        <v>1</v>
+      </c>
       <c r="T23" s="53"/>
       <c r="U23" s="48"/>
       <c r="V23" s="48"/>
@@ -10892,15 +10894,15 @@
       <c r="OM23" s="4"/>
       <c r="ON23" s="4"/>
     </row>
-    <row r="24" spans="1:410" s="1" customFormat="1" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:410" s="1" customFormat="1" ht="12.95" customHeight="1" thickTop="1">
       <c r="A24" s="10"/>
-      <c r="B24" s="106" t="s">
-        <v>25</v>
+      <c r="B24" s="129" t="s">
+        <v>21</v>
       </c>
-      <c r="C24" s="106">
+      <c r="C24" s="129">
         <v>2</v>
       </c>
-      <c r="D24" s="106">
+      <c r="D24" s="129">
         <v>0</v>
       </c>
       <c r="E24" s="47"/>
@@ -11314,11 +11316,11 @@
       <c r="OS24" s="2"/>
       <c r="OT24" s="2"/>
     </row>
-    <row r="25" spans="1:410" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="105"/>
-      <c r="B25" s="107"/>
-      <c r="C25" s="107"/>
-      <c r="D25" s="107"/>
+    <row r="25" spans="1:410" ht="12.95" customHeight="1" thickBot="1">
+      <c r="A25" s="141"/>
+      <c r="B25" s="130"/>
+      <c r="C25" s="130"/>
+      <c r="D25" s="130"/>
       <c r="E25" s="47"/>
       <c r="F25" s="47"/>
       <c r="G25" s="47"/>
@@ -11333,8 +11335,12 @@
       <c r="P25" s="48"/>
       <c r="Q25" s="53"/>
       <c r="R25" s="53"/>
-      <c r="S25" s="53"/>
-      <c r="T25" s="53"/>
+      <c r="S25" s="106">
+        <v>2</v>
+      </c>
+      <c r="T25" s="106">
+        <v>1</v>
+      </c>
       <c r="U25" s="48"/>
       <c r="V25" s="48"/>
       <c r="W25" s="48"/>
@@ -11720,10 +11726,10 @@
       <c r="OM25" s="4"/>
       <c r="ON25" s="4"/>
     </row>
-    <row r="26" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="105"/>
+    <row r="26" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A26" s="141"/>
       <c r="B26" s="60" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="C26" s="36"/>
       <c r="D26" s="37"/>
@@ -12128,15 +12134,15 @@
       <c r="OM26" s="4"/>
       <c r="ON26" s="4"/>
     </row>
-    <row r="27" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="105"/>
-      <c r="B27" s="120" t="s">
-        <v>28</v>
+    <row r="27" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A27" s="141"/>
+      <c r="B27" s="128" t="s">
+        <v>23</v>
       </c>
-      <c r="C27" s="119">
+      <c r="C27" s="127">
         <v>3</v>
       </c>
-      <c r="D27" s="119">
+      <c r="D27" s="127">
         <v>0</v>
       </c>
       <c r="E27" s="47"/>
@@ -12544,11 +12550,11 @@
       <c r="OM27" s="4"/>
       <c r="ON27" s="4"/>
     </row>
-    <row r="28" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="105"/>
-      <c r="B28" s="120"/>
-      <c r="C28" s="119"/>
-      <c r="D28" s="119"/>
+    <row r="28" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A28" s="141"/>
+      <c r="B28" s="128"/>
+      <c r="C28" s="127"/>
+      <c r="D28" s="127"/>
       <c r="E28" s="47"/>
       <c r="F28" s="47"/>
       <c r="G28" s="47"/>
@@ -12950,15 +12956,15 @@
       <c r="OM28" s="4"/>
       <c r="ON28" s="4"/>
     </row>
-    <row r="29" spans="1:410" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="105"/>
-      <c r="B29" s="109" t="s">
-        <v>27</v>
+    <row r="29" spans="1:410" ht="12.95" customHeight="1" thickTop="1">
+      <c r="A29" s="141"/>
+      <c r="B29" s="131" t="s">
+        <v>24</v>
       </c>
-      <c r="C29" s="109">
+      <c r="C29" s="131">
         <v>2</v>
       </c>
-      <c r="D29" s="109">
+      <c r="D29" s="131">
         <v>0</v>
       </c>
       <c r="E29" s="47"/>
@@ -13364,11 +13370,11 @@
       <c r="OM29" s="4"/>
       <c r="ON29" s="4"/>
     </row>
-    <row r="30" spans="1:410" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="105"/>
-      <c r="B30" s="110"/>
-      <c r="C30" s="110"/>
-      <c r="D30" s="110"/>
+    <row r="30" spans="1:410" ht="12.95" customHeight="1" thickBot="1">
+      <c r="A30" s="141"/>
+      <c r="B30" s="132"/>
+      <c r="C30" s="132"/>
+      <c r="D30" s="132"/>
       <c r="E30" s="47"/>
       <c r="F30" s="47"/>
       <c r="G30" s="47"/>
@@ -13770,15 +13776,15 @@
       <c r="OM30" s="4"/>
       <c r="ON30" s="4"/>
     </row>
-    <row r="31" spans="1:410" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="105"/>
-      <c r="B31" s="109" t="s">
-        <v>31</v>
+    <row r="31" spans="1:410" ht="12.95" customHeight="1" thickTop="1">
+      <c r="A31" s="141"/>
+      <c r="B31" s="131" t="s">
+        <v>25</v>
       </c>
-      <c r="C31" s="109">
+      <c r="C31" s="131">
         <v>3</v>
       </c>
-      <c r="D31" s="109">
+      <c r="D31" s="131">
         <v>0</v>
       </c>
       <c r="E31" s="47"/>
@@ -14186,11 +14192,11 @@
       <c r="OM31" s="4"/>
       <c r="ON31" s="4"/>
     </row>
-    <row r="32" spans="1:410" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="105"/>
-      <c r="B32" s="110"/>
-      <c r="C32" s="110"/>
-      <c r="D32" s="110"/>
+    <row r="32" spans="1:410" ht="12.95" customHeight="1" thickBot="1">
+      <c r="A32" s="141"/>
+      <c r="B32" s="132"/>
+      <c r="C32" s="132"/>
+      <c r="D32" s="132"/>
       <c r="E32" s="47"/>
       <c r="F32" s="47"/>
       <c r="G32" s="47"/>
@@ -14592,15 +14598,15 @@
       <c r="OM32" s="4"/>
       <c r="ON32" s="4"/>
     </row>
-    <row r="33" spans="1:410" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="105"/>
-      <c r="B33" s="109" t="s">
-        <v>33</v>
+    <row r="33" spans="1:410" ht="12.95" customHeight="1" thickTop="1">
+      <c r="A33" s="141"/>
+      <c r="B33" s="131" t="s">
+        <v>26</v>
       </c>
-      <c r="C33" s="109">
+      <c r="C33" s="131">
         <v>2</v>
       </c>
-      <c r="D33" s="109">
+      <c r="D33" s="131">
         <v>0</v>
       </c>
       <c r="E33" s="47"/>
@@ -15008,11 +15014,11 @@
       <c r="OM33" s="4"/>
       <c r="ON33" s="4"/>
     </row>
-    <row r="34" spans="1:410" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="105"/>
-      <c r="B34" s="110"/>
-      <c r="C34" s="110"/>
-      <c r="D34" s="110"/>
+    <row r="34" spans="1:410" ht="12.95" customHeight="1" thickBot="1">
+      <c r="A34" s="141"/>
+      <c r="B34" s="132"/>
+      <c r="C34" s="132"/>
+      <c r="D34" s="132"/>
       <c r="E34" s="47"/>
       <c r="F34" s="47"/>
       <c r="G34" s="47"/>
@@ -15414,10 +15420,10 @@
       <c r="OM34" s="4"/>
       <c r="ON34" s="4"/>
     </row>
-    <row r="35" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="105"/>
+    <row r="35" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A35" s="141"/>
       <c r="B35" s="61" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="C35" s="32"/>
       <c r="D35" s="33"/>
@@ -15824,15 +15830,15 @@
       <c r="OM35" s="4"/>
       <c r="ON35" s="4"/>
     </row>
-    <row r="36" spans="1:410" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="105"/>
-      <c r="B36" s="113" t="s">
-        <v>5</v>
+    <row r="36" spans="1:410" ht="12.95" customHeight="1" thickTop="1">
+      <c r="A36" s="141"/>
+      <c r="B36" s="133" t="s">
+        <v>28</v>
       </c>
-      <c r="C36" s="113">
+      <c r="C36" s="133">
         <v>3</v>
       </c>
-      <c r="D36" s="113">
+      <c r="D36" s="133">
         <v>0</v>
       </c>
       <c r="E36" s="47"/>
@@ -16240,11 +16246,11 @@
       <c r="OM36" s="4"/>
       <c r="ON36" s="4"/>
     </row>
-    <row r="37" spans="1:410" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="105"/>
-      <c r="B37" s="114"/>
-      <c r="C37" s="114"/>
-      <c r="D37" s="114"/>
+    <row r="37" spans="1:410" ht="12.95" customHeight="1" thickBot="1">
+      <c r="A37" s="141"/>
+      <c r="B37" s="134"/>
+      <c r="C37" s="134"/>
+      <c r="D37" s="134"/>
       <c r="E37" s="47"/>
       <c r="F37" s="47"/>
       <c r="G37" s="47"/>
@@ -16646,10 +16652,10 @@
       <c r="OM37" s="4"/>
       <c r="ON37" s="4"/>
     </row>
-    <row r="38" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="105"/>
+    <row r="38" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A38" s="141"/>
       <c r="B38" s="61" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="C38" s="32"/>
       <c r="D38" s="33"/>
@@ -17054,15 +17060,15 @@
       <c r="OM38" s="4"/>
       <c r="ON38" s="4"/>
     </row>
-    <row r="39" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="105"/>
-      <c r="B39" s="112" t="s">
-        <v>35</v>
+    <row r="39" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A39" s="141"/>
+      <c r="B39" s="140" t="s">
+        <v>30</v>
       </c>
-      <c r="C39" s="111">
+      <c r="C39" s="139">
         <v>7</v>
       </c>
-      <c r="D39" s="111">
+      <c r="D39" s="139">
         <v>0</v>
       </c>
       <c r="E39" s="47"/>
@@ -17474,11 +17480,11 @@
       <c r="OM39" s="4"/>
       <c r="ON39" s="4"/>
     </row>
-    <row r="40" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="105"/>
-      <c r="B40" s="112"/>
-      <c r="C40" s="111"/>
-      <c r="D40" s="111"/>
+    <row r="40" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A40" s="141"/>
+      <c r="B40" s="140"/>
+      <c r="C40" s="139"/>
+      <c r="D40" s="139"/>
       <c r="E40" s="47"/>
       <c r="F40" s="47"/>
       <c r="G40" s="47"/>
@@ -17880,15 +17886,15 @@
       <c r="OM40" s="4"/>
       <c r="ON40" s="4"/>
     </row>
-    <row r="41" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="105"/>
-      <c r="B41" s="112" t="s">
-        <v>36</v>
+    <row r="41" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A41" s="141"/>
+      <c r="B41" s="140" t="s">
+        <v>31</v>
       </c>
-      <c r="C41" s="111">
+      <c r="C41" s="139">
         <v>11</v>
       </c>
-      <c r="D41" s="111">
+      <c r="D41" s="139">
         <v>0</v>
       </c>
       <c r="E41" s="47"/>
@@ -18304,11 +18310,11 @@
       <c r="OM41" s="4"/>
       <c r="ON41" s="4"/>
     </row>
-    <row r="42" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="105"/>
-      <c r="B42" s="112"/>
-      <c r="C42" s="111"/>
-      <c r="D42" s="111"/>
+    <row r="42" spans="1:410" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A42" s="141"/>
+      <c r="B42" s="140"/>
+      <c r="C42" s="139"/>
+      <c r="D42" s="139"/>
       <c r="E42" s="47"/>
       <c r="F42" s="47"/>
       <c r="G42" s="47"/>
@@ -18710,15 +18716,15 @@
       <c r="OM42" s="4"/>
       <c r="ON42" s="4"/>
     </row>
-    <row r="43" spans="1:410" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="105"/>
-      <c r="B43" s="117" t="s">
-        <v>37</v>
+    <row r="43" spans="1:410" ht="12.95" customHeight="1" thickTop="1">
+      <c r="A43" s="141"/>
+      <c r="B43" s="137" t="s">
+        <v>32</v>
       </c>
-      <c r="C43" s="115">
+      <c r="C43" s="135">
         <v>3</v>
       </c>
-      <c r="D43" s="115">
+      <c r="D43" s="135">
         <v>0</v>
       </c>
       <c r="E43" s="47"/>
@@ -19126,11 +19132,11 @@
       <c r="OM43" s="4"/>
       <c r="ON43" s="4"/>
     </row>
-    <row r="44" spans="1:410" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="105"/>
-      <c r="B44" s="118"/>
-      <c r="C44" s="116"/>
-      <c r="D44" s="116"/>
+    <row r="44" spans="1:410" ht="12.95" customHeight="1" thickBot="1">
+      <c r="A44" s="141"/>
+      <c r="B44" s="138"/>
+      <c r="C44" s="136"/>
+      <c r="D44" s="136"/>
       <c r="E44" s="47"/>
       <c r="F44" s="47"/>
       <c r="G44" s="47"/>
@@ -19532,15 +19538,15 @@
       <c r="OM44" s="4"/>
       <c r="ON44" s="4"/>
     </row>
-    <row r="45" spans="1:410" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="105"/>
-      <c r="B45" s="117" t="s">
-        <v>38</v>
+    <row r="45" spans="1:410" ht="12.95" customHeight="1" thickTop="1">
+      <c r="A45" s="141"/>
+      <c r="B45" s="137" t="s">
+        <v>33</v>
       </c>
-      <c r="C45" s="115">
+      <c r="C45" s="135">
         <v>3</v>
       </c>
-      <c r="D45" s="115">
+      <c r="D45" s="135">
         <v>0</v>
       </c>
       <c r="E45" s="47"/>
@@ -19948,11 +19954,11 @@
       <c r="OM45" s="4"/>
       <c r="ON45" s="4"/>
     </row>
-    <row r="46" spans="1:410" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="105"/>
-      <c r="B46" s="118"/>
-      <c r="C46" s="116"/>
-      <c r="D46" s="116"/>
+    <row r="46" spans="1:410" ht="12.95" customHeight="1" thickBot="1">
+      <c r="A46" s="141"/>
+      <c r="B46" s="138"/>
+      <c r="C46" s="136"/>
+      <c r="D46" s="136"/>
       <c r="E46" s="47"/>
       <c r="F46" s="47"/>
       <c r="G46" s="47"/>
@@ -20354,15 +20360,15 @@
       <c r="OM46" s="4"/>
       <c r="ON46" s="4"/>
     </row>
-    <row r="47" spans="1:410" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:410" ht="12.95" customHeight="1" thickTop="1">
       <c r="A47" s="10"/>
-      <c r="B47" s="117" t="s">
-        <v>40</v>
+      <c r="B47" s="137" t="s">
+        <v>34</v>
       </c>
-      <c r="C47" s="115">
+      <c r="C47" s="135">
         <v>3</v>
       </c>
-      <c r="D47" s="115">
+      <c r="D47" s="135">
         <v>0</v>
       </c>
       <c r="E47" s="47"/>
@@ -20776,11 +20782,11 @@
       <c r="OS47" s="46"/>
       <c r="OT47" s="46"/>
     </row>
-    <row r="48" spans="1:410" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:410" ht="12.95" customHeight="1" thickBot="1">
       <c r="A48" s="10"/>
-      <c r="B48" s="118"/>
-      <c r="C48" s="116"/>
-      <c r="D48" s="116"/>
+      <c r="B48" s="138"/>
+      <c r="C48" s="136"/>
+      <c r="D48" s="136"/>
       <c r="E48" s="47"/>
       <c r="F48" s="47"/>
       <c r="G48" s="47"/>
@@ -21188,15 +21194,15 @@
       <c r="OS48" s="46"/>
       <c r="OT48" s="46"/>
     </row>
-    <row r="49" spans="1:404" s="46" customFormat="1" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="105"/>
-      <c r="B49" s="117" t="s">
-        <v>39</v>
+    <row r="49" spans="1:404" s="46" customFormat="1" ht="12.95" customHeight="1" thickTop="1">
+      <c r="A49" s="141"/>
+      <c r="B49" s="137" t="s">
+        <v>35</v>
       </c>
-      <c r="C49" s="115">
+      <c r="C49" s="135">
         <v>3</v>
       </c>
-      <c r="D49" s="115">
+      <c r="D49" s="135">
         <v>0</v>
       </c>
       <c r="E49" s="47"/>
@@ -21604,11 +21610,11 @@
       <c r="OM49" s="45"/>
       <c r="ON49" s="45"/>
     </row>
-    <row r="50" spans="1:404" s="46" customFormat="1" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="105"/>
-      <c r="B50" s="118"/>
-      <c r="C50" s="116"/>
-      <c r="D50" s="116"/>
+    <row r="50" spans="1:404" s="46" customFormat="1" ht="12.95" customHeight="1" thickBot="1">
+      <c r="A50" s="141"/>
+      <c r="B50" s="138"/>
+      <c r="C50" s="136"/>
+      <c r="D50" s="136"/>
       <c r="E50" s="47"/>
       <c r="F50" s="47"/>
       <c r="G50" s="47"/>
@@ -22010,10 +22016,10 @@
       <c r="OM50" s="45"/>
       <c r="ON50" s="45"/>
     </row>
-    <row r="51" spans="1:404" s="46" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="105"/>
+    <row r="51" spans="1:404" s="46" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A51" s="141"/>
       <c r="B51" s="61" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="C51" s="32"/>
       <c r="D51" s="33"/>
@@ -22418,15 +22424,15 @@
       <c r="OM51" s="45"/>
       <c r="ON51" s="45"/>
     </row>
-    <row r="52" spans="1:404" s="46" customFormat="1" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="105"/>
-      <c r="B52" s="108" t="s">
-        <v>8</v>
+    <row r="52" spans="1:404" s="46" customFormat="1" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A52" s="141"/>
+      <c r="B52" s="112" t="s">
+        <v>37</v>
       </c>
-      <c r="C52" s="108">
+      <c r="C52" s="112">
         <v>5</v>
       </c>
-      <c r="D52" s="108">
+      <c r="D52" s="112">
         <v>0</v>
       </c>
       <c r="E52" s="47"/>
@@ -22836,11 +22842,11 @@
       <c r="OM52" s="45"/>
       <c r="ON52" s="45"/>
     </row>
-    <row r="53" spans="1:404" s="46" customFormat="1" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="105"/>
-      <c r="B53" s="108"/>
-      <c r="C53" s="108"/>
-      <c r="D53" s="108"/>
+    <row r="53" spans="1:404" s="46" customFormat="1" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A53" s="141"/>
+      <c r="B53" s="112"/>
+      <c r="C53" s="112"/>
+      <c r="D53" s="112"/>
       <c r="E53" s="47"/>
       <c r="F53" s="47"/>
       <c r="G53" s="47"/>
@@ -23242,15 +23248,15 @@
       <c r="OM53" s="45"/>
       <c r="ON53" s="45"/>
     </row>
-    <row r="54" spans="1:404" s="18" customFormat="1" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="105"/>
-      <c r="B54" s="108" t="s">
-        <v>9</v>
+    <row r="54" spans="1:404" s="18" customFormat="1" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A54" s="141"/>
+      <c r="B54" s="112" t="s">
+        <v>38</v>
       </c>
-      <c r="C54" s="108">
+      <c r="C54" s="112">
         <v>3</v>
       </c>
-      <c r="D54" s="108">
+      <c r="D54" s="112">
         <v>0</v>
       </c>
       <c r="E54" s="47"/>
@@ -23658,11 +23664,11 @@
       <c r="OM54" s="17"/>
       <c r="ON54" s="17"/>
     </row>
-    <row r="55" spans="1:404" s="10" customFormat="1" ht="12.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:404" s="10" customFormat="1" ht="12.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A55" s="13"/>
-      <c r="B55" s="108"/>
-      <c r="C55" s="108"/>
-      <c r="D55" s="108"/>
+      <c r="B55" s="112"/>
+      <c r="C55" s="112"/>
+      <c r="D55" s="112"/>
       <c r="E55" s="47"/>
       <c r="F55" s="47"/>
       <c r="G55" s="47"/>
@@ -24064,9 +24070,9 @@
       <c r="OM55" s="14"/>
       <c r="ON55" s="14"/>
     </row>
-    <row r="56" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="B56" s="61" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C56" s="32"/>
       <c r="D56" s="33"/>
@@ -24471,14 +24477,14 @@
       <c r="OM56" s="14"/>
       <c r="ON56" s="14"/>
     </row>
-    <row r="57" spans="1:404" s="10" customFormat="1" ht="12.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="136" t="s">
-        <v>11</v>
+    <row r="57" spans="1:404" s="10" customFormat="1" ht="12.95" customHeight="1" thickTop="1">
+      <c r="B57" s="110" t="s">
+        <v>40</v>
       </c>
-      <c r="C57" s="136">
+      <c r="C57" s="110">
         <v>3</v>
       </c>
-      <c r="D57" s="136">
+      <c r="D57" s="110">
         <v>0</v>
       </c>
       <c r="E57" s="47"/>
@@ -24886,10 +24892,10 @@
       <c r="OM57" s="14"/>
       <c r="ON57" s="14"/>
     </row>
-    <row r="58" spans="1:404" s="10" customFormat="1" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="137"/>
-      <c r="C58" s="137"/>
-      <c r="D58" s="137"/>
+    <row r="58" spans="1:404" s="10" customFormat="1" ht="12.95" customHeight="1" thickBot="1">
+      <c r="B58" s="111"/>
+      <c r="C58" s="111"/>
+      <c r="D58" s="111"/>
       <c r="E58" s="51"/>
       <c r="F58" s="51"/>
       <c r="G58" s="51"/>
@@ -25291,7 +25297,7 @@
       <c r="OM58" s="14"/>
       <c r="ON58" s="14"/>
     </row>
-    <row r="59" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="B59" s="64"/>
       <c r="C59" s="65"/>
       <c r="D59" s="66"/>
@@ -25696,9 +25702,9 @@
       <c r="OM59" s="14"/>
       <c r="ON59" s="14"/>
     </row>
-    <row r="60" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="B60" s="63" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C60" s="63">
         <f>SUM(C5:C58)</f>
@@ -26109,7 +26115,7 @@
       <c r="OM60" s="14"/>
       <c r="ON60" s="14"/>
     </row>
-    <row r="61" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" thickTop="1">
       <c r="D61" s="13"/>
       <c r="E61" s="13"/>
       <c r="F61" s="13"/>
@@ -26512,7 +26518,7 @@
       <c r="OM61" s="14"/>
       <c r="ON61" s="14"/>
     </row>
-    <row r="62" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="D62" s="13"/>
       <c r="E62" s="13"/>
       <c r="F62" s="13"/>
@@ -26915,7 +26921,7 @@
       <c r="OM62" s="14"/>
       <c r="ON62" s="14"/>
     </row>
-    <row r="63" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="C63"/>
       <c r="D63" s="13"/>
       <c r="E63" s="13"/>
@@ -27319,7 +27325,7 @@
       <c r="OM63" s="14"/>
       <c r="ON63" s="14"/>
     </row>
-    <row r="64" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="D64" s="13"/>
       <c r="E64" s="13"/>
       <c r="F64" s="13"/>
@@ -27722,7 +27728,7 @@
       <c r="OM64" s="14"/>
       <c r="ON64" s="14"/>
     </row>
-    <row r="65" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="C65"/>
       <c r="D65" s="13"/>
       <c r="E65" s="13"/>
@@ -28126,7 +28132,7 @@
       <c r="OM65" s="14"/>
       <c r="ON65" s="14"/>
     </row>
-    <row r="66" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="D66" s="13"/>
       <c r="E66" s="13"/>
       <c r="F66" s="13"/>
@@ -28529,7 +28535,7 @@
       <c r="OM66" s="14"/>
       <c r="ON66" s="14"/>
     </row>
-    <row r="67" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="C67" s="13"/>
       <c r="D67" s="13"/>
       <c r="E67" s="13"/>
@@ -28933,7 +28939,7 @@
       <c r="OM67" s="14"/>
       <c r="ON67" s="14"/>
     </row>
-    <row r="68" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="C68" s="13"/>
       <c r="D68" s="13"/>
       <c r="E68" s="13"/>
@@ -29337,7 +29343,7 @@
       <c r="OM68" s="14"/>
       <c r="ON68" s="14"/>
     </row>
-    <row r="69" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="C69" s="13"/>
       <c r="D69" s="13"/>
       <c r="E69" s="13"/>
@@ -29741,7 +29747,7 @@
       <c r="OM69" s="14"/>
       <c r="ON69" s="14"/>
     </row>
-    <row r="70" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="C70" s="13"/>
       <c r="D70" s="13"/>
       <c r="E70" s="13"/>
@@ -30145,7 +30151,7 @@
       <c r="OM70" s="14"/>
       <c r="ON70" s="14"/>
     </row>
-    <row r="71" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="AS71" s="13"/>
       <c r="AT71" s="13"/>
       <c r="AU71" s="13"/>
@@ -30507,7 +30513,7 @@
       <c r="OM71" s="14"/>
       <c r="ON71" s="14"/>
     </row>
-    <row r="72" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="AS72" s="13"/>
       <c r="AT72" s="13"/>
       <c r="AU72" s="13"/>
@@ -30869,7 +30875,7 @@
       <c r="OM72" s="14"/>
       <c r="ON72" s="14"/>
     </row>
-    <row r="73" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="AS73" s="13"/>
       <c r="AT73" s="13"/>
       <c r="AU73" s="13"/>
@@ -31231,7 +31237,7 @@
       <c r="OM73" s="14"/>
       <c r="ON73" s="14"/>
     </row>
-    <row r="74" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A74" s="13"/>
       <c r="AS74" s="13"/>
       <c r="AT74" s="13"/>
@@ -31594,7 +31600,7 @@
       <c r="OM74" s="14"/>
       <c r="ON74" s="14"/>
     </row>
-    <row r="75" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A75" s="13"/>
       <c r="AS75" s="13"/>
       <c r="AT75" s="13"/>
@@ -31957,7 +31963,7 @@
       <c r="OM75" s="14"/>
       <c r="ON75" s="14"/>
     </row>
-    <row r="76" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A76" s="13"/>
       <c r="AS76" s="14"/>
       <c r="AT76" s="14"/>
@@ -32320,7 +32326,7 @@
       <c r="OM76" s="14"/>
       <c r="ON76" s="14"/>
     </row>
-    <row r="77" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A77" s="13"/>
       <c r="AS77" s="14"/>
       <c r="AT77" s="14"/>
@@ -32683,7 +32689,7 @@
       <c r="OM77" s="14"/>
       <c r="ON77" s="14"/>
     </row>
-    <row r="78" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A78" s="13"/>
       <c r="AS78" s="14"/>
       <c r="AT78" s="14"/>
@@ -33046,7 +33052,7 @@
       <c r="OM78" s="14"/>
       <c r="ON78" s="14"/>
     </row>
-    <row r="79" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A79" s="13"/>
       <c r="AS79" s="14"/>
       <c r="AT79" s="14"/>
@@ -33409,7 +33415,7 @@
       <c r="OM79" s="14"/>
       <c r="ON79" s="14"/>
     </row>
-    <row r="80" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A80" s="13"/>
       <c r="AS80" s="14"/>
       <c r="AT80" s="14"/>
@@ -33772,7 +33778,7 @@
       <c r="OM80" s="14"/>
       <c r="ON80" s="14"/>
     </row>
-    <row r="81" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A81" s="13"/>
       <c r="AS81" s="14"/>
       <c r="AT81" s="14"/>
@@ -34135,7 +34141,7 @@
       <c r="OM81" s="14"/>
       <c r="ON81" s="14"/>
     </row>
-    <row r="82" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A82" s="13"/>
       <c r="AS82" s="14"/>
       <c r="AT82" s="14"/>
@@ -34498,7 +34504,7 @@
       <c r="OM82" s="14"/>
       <c r="ON82" s="14"/>
     </row>
-    <row r="83" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A83" s="13"/>
       <c r="AS83" s="14"/>
       <c r="AT83" s="14"/>
@@ -34861,7 +34867,7 @@
       <c r="OM83" s="14"/>
       <c r="ON83" s="14"/>
     </row>
-    <row r="84" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A84" s="13"/>
       <c r="AS84" s="14"/>
       <c r="AT84" s="14"/>
@@ -35224,7 +35230,7 @@
       <c r="OM84" s="14"/>
       <c r="ON84" s="14"/>
     </row>
-    <row r="85" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A85" s="13"/>
       <c r="AS85" s="14"/>
       <c r="AT85" s="14"/>
@@ -35587,7 +35593,7 @@
       <c r="OM85" s="14"/>
       <c r="ON85" s="14"/>
     </row>
-    <row r="86" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A86" s="13"/>
       <c r="AS86" s="14"/>
       <c r="AT86" s="14"/>
@@ -35950,7 +35956,7 @@
       <c r="OM86" s="14"/>
       <c r="ON86" s="14"/>
     </row>
-    <row r="87" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A87" s="13"/>
       <c r="AS87" s="14"/>
       <c r="AT87" s="14"/>
@@ -36313,7 +36319,7 @@
       <c r="OM87" s="14"/>
       <c r="ON87" s="14"/>
     </row>
-    <row r="88" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A88" s="13"/>
       <c r="AS88" s="14"/>
       <c r="AT88" s="14"/>
@@ -36676,7 +36682,7 @@
       <c r="OM88" s="14"/>
       <c r="ON88" s="14"/>
     </row>
-    <row r="89" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A89" s="13"/>
       <c r="AS89" s="14"/>
       <c r="AT89" s="14"/>
@@ -37039,7 +37045,7 @@
       <c r="OM89" s="14"/>
       <c r="ON89" s="14"/>
     </row>
-    <row r="90" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A90" s="13"/>
       <c r="AS90" s="14"/>
       <c r="AT90" s="14"/>
@@ -37402,7 +37408,7 @@
       <c r="OM90" s="14"/>
       <c r="ON90" s="14"/>
     </row>
-    <row r="91" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A91" s="13"/>
       <c r="AS91" s="14"/>
       <c r="AT91" s="14"/>
@@ -37765,7 +37771,7 @@
       <c r="OM91" s="14"/>
       <c r="ON91" s="14"/>
     </row>
-    <row r="92" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A92" s="13"/>
       <c r="AS92" s="14"/>
       <c r="AT92" s="14"/>
@@ -38128,7 +38134,7 @@
       <c r="OM92" s="14"/>
       <c r="ON92" s="14"/>
     </row>
-    <row r="93" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A93" s="13"/>
       <c r="AS93" s="14"/>
       <c r="AT93" s="14"/>
@@ -38491,7 +38497,7 @@
       <c r="OM93" s="14"/>
       <c r="ON93" s="14"/>
     </row>
-    <row r="94" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A94" s="13"/>
       <c r="AS94" s="14"/>
       <c r="AT94" s="14"/>
@@ -38854,7 +38860,7 @@
       <c r="OM94" s="14"/>
       <c r="ON94" s="14"/>
     </row>
-    <row r="95" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A95" s="13"/>
       <c r="AS95" s="14"/>
       <c r="AT95" s="14"/>
@@ -39217,7 +39223,7 @@
       <c r="OM95" s="14"/>
       <c r="ON95" s="14"/>
     </row>
-    <row r="96" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A96" s="13"/>
       <c r="AS96" s="14"/>
       <c r="AT96" s="14"/>
@@ -39580,7 +39586,7 @@
       <c r="OM96" s="14"/>
       <c r="ON96" s="14"/>
     </row>
-    <row r="97" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A97" s="13"/>
       <c r="AS97" s="14"/>
       <c r="AT97" s="14"/>
@@ -39943,7 +39949,7 @@
       <c r="OM97" s="14"/>
       <c r="ON97" s="14"/>
     </row>
-    <row r="98" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A98" s="13"/>
       <c r="AS98" s="14"/>
       <c r="AT98" s="14"/>
@@ -40306,7 +40312,7 @@
       <c r="OM98" s="14"/>
       <c r="ON98" s="14"/>
     </row>
-    <row r="99" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A99" s="13"/>
       <c r="AS99" s="14"/>
       <c r="AT99" s="14"/>
@@ -40669,7 +40675,7 @@
       <c r="OM99" s="14"/>
       <c r="ON99" s="14"/>
     </row>
-    <row r="100" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A100" s="13"/>
       <c r="AS100" s="14"/>
       <c r="AT100" s="14"/>
@@ -41032,7 +41038,7 @@
       <c r="OM100" s="14"/>
       <c r="ON100" s="14"/>
     </row>
-    <row r="101" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A101" s="13"/>
       <c r="AS101" s="14"/>
       <c r="AT101" s="14"/>
@@ -41395,7 +41401,7 @@
       <c r="OM101" s="14"/>
       <c r="ON101" s="14"/>
     </row>
-    <row r="102" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A102" s="13"/>
       <c r="AS102" s="14"/>
       <c r="AT102" s="14"/>
@@ -41758,7 +41764,7 @@
       <c r="OM102" s="14"/>
       <c r="ON102" s="14"/>
     </row>
-    <row r="103" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A103" s="13"/>
       <c r="AS103" s="14"/>
       <c r="AT103" s="14"/>
@@ -42121,7 +42127,7 @@
       <c r="OM103" s="14"/>
       <c r="ON103" s="14"/>
     </row>
-    <row r="104" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A104" s="13"/>
       <c r="AS104" s="14"/>
       <c r="AT104" s="14"/>
@@ -42484,7 +42490,7 @@
       <c r="OM104" s="14"/>
       <c r="ON104" s="14"/>
     </row>
-    <row r="105" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A105" s="13"/>
       <c r="AS105" s="14"/>
       <c r="AT105" s="14"/>
@@ -42847,7 +42853,7 @@
       <c r="OM105" s="14"/>
       <c r="ON105" s="14"/>
     </row>
-    <row r="106" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A106" s="13"/>
       <c r="AS106" s="14"/>
       <c r="AT106" s="14"/>
@@ -43210,7 +43216,7 @@
       <c r="OM106" s="14"/>
       <c r="ON106" s="14"/>
     </row>
-    <row r="107" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A107" s="13"/>
       <c r="AS107" s="14"/>
       <c r="AT107" s="14"/>
@@ -43573,7 +43579,7 @@
       <c r="OM107" s="14"/>
       <c r="ON107" s="14"/>
     </row>
-    <row r="108" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A108" s="13"/>
       <c r="AS108" s="14"/>
       <c r="AT108" s="14"/>
@@ -43936,7 +43942,7 @@
       <c r="OM108" s="14"/>
       <c r="ON108" s="14"/>
     </row>
-    <row r="109" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A109" s="13"/>
       <c r="AS109" s="14"/>
       <c r="AT109" s="14"/>
@@ -44299,7 +44305,7 @@
       <c r="OM109" s="14"/>
       <c r="ON109" s="14"/>
     </row>
-    <row r="110" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A110" s="13"/>
       <c r="AS110" s="14"/>
       <c r="AT110" s="14"/>
@@ -44662,7 +44668,7 @@
       <c r="OM110" s="14"/>
       <c r="ON110" s="14"/>
     </row>
-    <row r="111" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A111" s="13"/>
       <c r="AS111" s="14"/>
       <c r="AT111" s="14"/>
@@ -45025,7 +45031,7 @@
       <c r="OM111" s="14"/>
       <c r="ON111" s="14"/>
     </row>
-    <row r="112" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:404" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A112" s="13"/>
       <c r="AS112" s="14"/>
       <c r="AT112" s="14"/>
@@ -45388,7 +45394,7 @@
       <c r="OM112" s="14"/>
       <c r="ON112" s="14"/>
     </row>
-    <row r="113" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A113" s="13"/>
       <c r="AS113" s="14"/>
       <c r="AT113" s="14"/>
@@ -45751,7 +45757,7 @@
       <c r="OM113" s="14"/>
       <c r="ON113" s="14"/>
     </row>
-    <row r="114" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A114" s="13"/>
       <c r="AS114" s="14"/>
       <c r="AT114" s="14"/>
@@ -46114,7 +46120,7 @@
       <c r="OM114" s="14"/>
       <c r="ON114" s="14"/>
     </row>
-    <row r="115" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A115" s="13"/>
       <c r="AS115" s="14"/>
       <c r="AT115" s="14"/>
@@ -46477,7 +46483,7 @@
       <c r="OM115" s="14"/>
       <c r="ON115" s="14"/>
     </row>
-    <row r="116" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A116" s="13"/>
       <c r="AS116" s="14"/>
       <c r="AT116" s="14"/>
@@ -46840,7 +46846,7 @@
       <c r="OM116" s="14"/>
       <c r="ON116" s="14"/>
     </row>
-    <row r="117" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A117" s="13"/>
       <c r="AS117" s="14"/>
       <c r="AT117" s="14"/>
@@ -47203,7 +47209,7 @@
       <c r="OM117" s="14"/>
       <c r="ON117" s="14"/>
     </row>
-    <row r="118" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A118" s="13"/>
       <c r="AS118" s="14"/>
       <c r="AT118" s="14"/>
@@ -47566,7 +47572,7 @@
       <c r="OM118" s="14"/>
       <c r="ON118" s="14"/>
     </row>
-    <row r="119" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A119" s="13"/>
       <c r="AS119" s="14"/>
       <c r="AT119" s="14"/>
@@ -47929,7 +47935,7 @@
       <c r="OM119" s="14"/>
       <c r="ON119" s="14"/>
     </row>
-    <row r="120" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A120" s="13"/>
       <c r="AS120" s="14"/>
       <c r="AT120" s="14"/>
@@ -48292,7 +48298,7 @@
       <c r="OM120" s="14"/>
       <c r="ON120" s="14"/>
     </row>
-    <row r="121" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A121" s="13"/>
       <c r="AS121" s="14"/>
       <c r="AT121" s="14"/>
@@ -48655,7 +48661,7 @@
       <c r="OM121" s="14"/>
       <c r="ON121" s="14"/>
     </row>
-    <row r="122" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A122" s="13"/>
       <c r="AS122" s="14"/>
       <c r="AT122" s="14"/>
@@ -49018,7 +49024,7 @@
       <c r="OM122" s="14"/>
       <c r="ON122" s="14"/>
     </row>
-    <row r="123" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1">
       <c r="A123" s="13"/>
       <c r="AS123" s="14"/>
       <c r="AT123" s="14"/>
@@ -49381,7 +49387,7 @@
       <c r="OM123" s="14"/>
       <c r="ON123" s="14"/>
     </row>
-    <row r="124" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:410" s="10" customFormat="1" ht="24.95" customHeight="1" thickBot="1">
       <c r="A124" s="34"/>
       <c r="AS124" s="11"/>
       <c r="AT124" s="11"/>
@@ -49750,7 +49756,7 @@
       <c r="OS124" s="12"/>
       <c r="OT124" s="12"/>
     </row>
-    <row r="125" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="B125" s="10"/>
       <c r="C125" s="10"/>
       <c r="D125" s="10"/>
@@ -50155,7 +50161,7 @@
       <c r="OM125" s="4"/>
       <c r="ON125" s="4"/>
     </row>
-    <row r="126" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="B126" s="10"/>
       <c r="C126" s="10"/>
       <c r="D126" s="10"/>
@@ -50560,7 +50566,7 @@
       <c r="OM126" s="4"/>
       <c r="ON126" s="4"/>
     </row>
-    <row r="127" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="B127" s="10"/>
       <c r="C127" s="10"/>
       <c r="D127" s="10"/>
@@ -50605,7 +50611,7 @@
       <c r="AQ127" s="10"/>
       <c r="AR127" s="10"/>
     </row>
-    <row r="128" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:410" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="B128" s="10"/>
       <c r="C128" s="10"/>
       <c r="D128" s="10"/>
@@ -50652,6 +50658,80 @@
     </row>
   </sheetData>
   <mergeCells count="90">
+    <mergeCell ref="A49:A54"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="A25:A46"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="D45:D46"/>
+    <mergeCell ref="A5:A12"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="AO2:AR2"/>
+    <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="U2:X2"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="A14:A19"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="AG2:AJ2"/>
+    <mergeCell ref="AK2:AN2"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
     <mergeCell ref="AT4:AU4"/>
     <mergeCell ref="AT3:AU3"/>
     <mergeCell ref="B57:B58"/>
@@ -50668,80 +50748,6 @@
     <mergeCell ref="D17:D18"/>
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="B15:B16"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="AG2:AJ2"/>
-    <mergeCell ref="AK2:AN2"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="AO2:AR2"/>
-    <mergeCell ref="Y2:AB2"/>
-    <mergeCell ref="A20:A23"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="M2:P2"/>
-    <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="U2:X2"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="A14:A19"/>
-    <mergeCell ref="A5:A12"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D47:D48"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="D45:D46"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="D41:D42"/>
-    <mergeCell ref="D39:D40"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="A49:A54"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="A25:A46"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C47:C48"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -50985,15 +50991,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <SharedWithUsers xmlns="f36c19d8-7c26-433c-b4f2-a48145021c82">
@@ -51012,46 +51009,23 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{533B2E84-B152-48FC-B211-FB1F29030CF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f36c19d8-7c26-433c-b4f2-a48145021c82"/>
-    <ds:schemaRef ds:uri="a52bb63a-e416-4320-b6d4-d17e553d625a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{533B2E84-B152-48FC-B211-FB1F29030CF7}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D77A291-D2C5-42CC-A6B7-E46687E08440}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E75F7AB-F066-41ED-A0B3-9FD20EED7FE2}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E75F7AB-F066-41ED-A0B3-9FD20EED7FE2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="f36c19d8-7c26-433c-b4f2-a48145021c82"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a52bb63a-e416-4320-b6d4-d17e553d625a"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D77A291-D2C5-42CC-A6B7-E46687E08440}"/>
 </file>
</xml_diff>